<commit_message>
Add U16 U17 groups and coach player notes
</commit_message>
<xml_diff>
--- a/public/templates/champion-import-game-activity.xlsx
+++ b/public/templates/champion-import-game-activity.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ігрова діяльність" sheetId="1" r:id="Ra29badd1562b46e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інструкція" sheetId="2" r:id="R7b12c17566444930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ігрова діяльність" sheetId="1" r:id="R9e84d980bb654248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інструкція" sheetId="2" r:id="Ra74e231253054458"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2008,7 +2008,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A2:A5001">
-      <x:formula1>"U6,U7,U8A,U8B,U9A,U9B,U10A,U10B,U11A,U11B,U12A,U12B,U13A,U13B,U14A,U14B,U15A,U15B,Воротарі A,Воротарі B,Воротарі C"</x:formula1>
+      <x:formula1>"U6,U7,U8A,U8B,U9A,U9B,U10A,U10B,U11A,U11B,U12A,U12B,U13A,U13B,U14A,U14B,U15A,U15B,U16A,U16B,U17A,U17B,Воротарі A,Воротарі B,Воротарі C"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>